<commit_message>
release: align bundled templates with v3.3 metadata
</commit_message>
<xml_diff>
--- a/templates/Weekflow_Task导入模板.xlsx
+++ b/templates/Weekflow_Task导入模板.xlsx
@@ -8,7 +8,7 @@
     <sheet name="填写说明" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Task导入!$A$4:$T$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Task导入!$A$4:$Z$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">进度历史!$A$4:$K$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2">填写说明!$A$7:$D$27</definedName>
   </definedNames>
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:Z4"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -426,6 +426,12 @@
     <col min="18" max="18" width="34.83203125" customWidth="1"/>
     <col min="19" max="19" width="38.83203125" customWidth="1"/>
     <col min="20" max="20" width="38.83203125" customWidth="1"/>
+    <col min="21" max="21" width="26.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="26.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="26.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="26.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="26.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="26.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,16 +510,34 @@
       <c r="T4" t="str">
         <v>交付物链接</v>
       </c>
+      <c r="U4" t="str">
+        <v>分组归档时间</v>
+      </c>
+      <c r="V4" t="str">
+        <v>分组归档批次</v>
+      </c>
+      <c r="W4" t="str">
+        <v>Flow归档时间</v>
+      </c>
+      <c r="X4" t="str">
+        <v>Flow归档批次</v>
+      </c>
+      <c r="Y4" t="str">
+        <v>Task归档时间</v>
+      </c>
+      <c r="Z4" t="str">
+        <v>Task归档批次</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:T4"/>
+  <autoFilter ref="A4:Z4"/>
   <mergeCells count="3">
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="A2:T2"/>
-    <mergeCell ref="A3:T3"/>
+    <mergeCell ref="A1:Z1"/>
+    <mergeCell ref="A2:Z2"/>
+    <mergeCell ref="A3:Z3"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>